<commit_message>
Set approved layout to compact (COMPARE_device1_compact_Card)
User approved compact 4-column layout as production default.
Regenerate TEST download files without № column or device strip.

Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/download/TEST_Daily_Report.xlsx
+++ b/equipment-templates/output/download/TEST_Daily_Report.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,18 +42,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
     <font>
@@ -67,7 +61,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -82,11 +76,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -184,7 +173,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -193,45 +182,39 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -599,38 +582,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>№</t>
+          <t>Поле</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Поле</t>
+          <t>Значение</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Значение</t>
+          <t>Ед.</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Отметка ✓/✗</t>
         </is>
@@ -639,205 +616,175 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>№ = пункт проверки  |  Жёлтые = ввод  |  Голубые = из базы  |  Отметка: ✓ / ✗ / 1-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
+          <t>Жёлтые ячейки — ввод вручную  |  Голубые — из базы  |  Отметка: ✓ / ✗ / 1-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Локация: Риелторы (Тюмень)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
+          <t>ЕЖЕДНЕВНЫЙ ОТЧЕТ О ХОДЕ ПЕРЕДАЧИ ДЕЛ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>ЕЖЕДНЕВНЫЙ ОТЧЕТ О ХОДЕ ПЕРЕДАЧИ ДЕЛ</t>
-        </is>
-      </c>
+          <t>Дата</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>23.06.2026</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="5" t="inlineStr"/>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Дата</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>22.06.2026</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr"/>
-      <c r="E5" s="9" t="inlineStr"/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Инженер</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Александр</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="5" t="inlineStr"/>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Инженер</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Александр</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr"/>
-      <c r="E6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7" ht="6" customHeight="1"/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>1. ЛОКАЦИЯ ДНЯ:</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Локация дня</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Риелторы (Тюмень)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+    </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>1. ЛОКАЦИЯ ДНЯ:</t>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>2. СТАТУС ПО ОЦЕНКАМ (сводка за день):</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="inlineStr"/>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Локация дня</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Риелторы (Тюмень)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr"/>
-      <c r="E9" s="9" t="inlineStr"/>
-    </row>
-    <row r="10" ht="6" customHeight="1"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>🟢 Оценка 4-5 (хорошее/отличное):</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>🟡 Оценка 3 (удовлетворительное):</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr"/>
+      <c r="C10" s="6" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
+    </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>2. СТАТУС ПО ОЦЕНКАМ (сводка за день):</t>
-        </is>
-      </c>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>🔴 Оценка 1-2 (требует внимания):</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr"/>
+      <c r="C11" s="6" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="5" t="inlineStr"/>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>🟢 Оценка 4-5 (хорошее/отличное):</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="8" t="inlineStr"/>
-      <c r="E12" s="9" t="inlineStr"/>
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>3. КРАСНЫЕ ФЛАГИ (эскалация Наталье):</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="5" t="inlineStr"/>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>🟡 Оценка 3 (удовлетворительное):</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="8" t="inlineStr"/>
-      <c r="E13" s="9" t="inlineStr"/>
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr"/>
+      <c r="C13" s="6" t="inlineStr"/>
+      <c r="D13" s="13" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="5" t="inlineStr"/>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>🔴 Оценка 1-2 (требует внимания):</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="8" t="inlineStr"/>
-      <c r="E14" s="9" t="inlineStr"/>
-    </row>
-    <row r="15" ht="6" customHeight="1"/>
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Да (кол-во: _____ шт.)</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr"/>
+      <c r="C14" s="6" t="inlineStr"/>
+      <c r="D14" s="13" t="inlineStr"/>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Краткое описание</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr"/>
+    </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>3. КРАСНЫЕ ФЛАГИ (эскалация Наталье):</t>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>4. ПРОБЛЕМЫ / БЛОКЕРЫ:</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Нет</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="inlineStr"/>
-      <c r="D17" s="8" t="inlineStr"/>
-      <c r="E17" s="15" t="inlineStr"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>5. ПЛАН НА ЗАВТРА:</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>Да (кол-во: _____ шт.)</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="inlineStr"/>
-      <c r="D18" s="8" t="inlineStr"/>
-      <c r="E18" s="15" t="inlineStr"/>
-    </row>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="5" t="inlineStr"/>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Краткое описание</t>
-        </is>
-      </c>
-      <c r="C19" s="16" t="inlineStr"/>
-    </row>
-    <row r="20" ht="6" customHeight="1"/>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>4. ПРОБЛЕМЫ / БЛОКЕРЫ:</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>5. ПЛАН НА ЗАВТРА:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="5" t="inlineStr"/>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Локация</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr"/>
-      <c r="D23" s="8" t="inlineStr"/>
-      <c r="E23" s="9" t="inlineStr"/>
+      <c r="B18" s="9" t="inlineStr"/>
+      <c r="C18" s="6" t="inlineStr"/>
+      <c r="D18" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A3:E3"/>
+  <mergeCells count="8">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E17 E18" showDropDown="1" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D13 D14" showDropDown="1" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓,✗,—"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>